<commit_message>
Update tower minimum weight and enhance productivity summary export functionality
- Changed `TOWER_MIN_MT` from 10.0 to 4.0 in `erection_compiled_to_daily_new.py` to adjust business rules.
- Added new functions in `workbook.py` to generate quarter week labels and assign quarter week buckets for improved productivity reporting.
- Enhanced the `export_erection_productivity_summary` function to support quarter-based data aggregation and improved review table generation.
- Updated multiple binary files to reflect recent changes in data processing.
</commit_message>
<xml_diff>
--- a/Raw Data/Projects and PCH.xlsx
+++ b/Raw Data/Projects and PCH.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2650736-72C0-438A-9774-5FB34DF5B1A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC4962EC-DE2F-4859-BF63-44B134DC520D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
   <si>
     <t>Mr. Sanjay Kumar Gupta</t>
   </si>
@@ -105,6 +105,12 @@
   </si>
   <si>
     <t>TA509</t>
+  </si>
+  <si>
+    <t>TA601</t>
+  </si>
+  <si>
+    <t>TB501</t>
   </si>
 </sst>
 </file>
@@ -655,11 +661,23 @@
       <c r="I18" s="2"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>23</v>
+      </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-01-29 16:10:20
</commit_message>
<xml_diff>
--- a/Raw Data/Projects and PCH.xlsx
+++ b/Raw Data/Projects and PCH.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC4962EC-DE2F-4859-BF63-44B134DC520D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21697C3-D18A-4A76-BD5C-D473CE37065F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
   <si>
     <t>Mr. Sanjay Kumar Gupta</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>TB501</t>
+  </si>
+  <si>
+    <t>Mr. Nabajit Baruah</t>
   </si>
 </sst>
 </file>
@@ -563,7 +566,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
@@ -574,7 +577,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
@@ -585,7 +588,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Apply dashboard updates without bulky pipeline history
</commit_message>
<xml_diff>
--- a/Raw Data/Projects and PCH.xlsx
+++ b/Raw Data/Projects and PCH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AFF9298-8F93-4FBA-A427-01A2A19156BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8685DFE4-3928-421D-A612-A0FDBFED415D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="32">
-  <si>
-    <t>Mr. Sanjay Kumar Gupta</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="31">
   <si>
     <t>TA413</t>
   </si>
@@ -95,9 +92,6 @@
     <t>Project Name</t>
   </si>
   <si>
-    <t>Mr. Dheeraj Vashishth</t>
-  </si>
-  <si>
     <t>TA513</t>
   </si>
   <si>
@@ -135,6 +129,9 @@
   </si>
   <si>
     <t>TA310</t>
+  </si>
+  <si>
+    <t>Mr. NK Gupta</t>
   </si>
 </sst>
 </file>
@@ -169,6 +166,7 @@
       <sz val="11"/>
       <color rgb="FF111827"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -522,39 +520,39 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="7"/>
@@ -562,13 +560,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="6"/>
@@ -576,13 +574,13 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="7"/>
@@ -590,13 +588,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="6"/>
@@ -604,13 +602,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="7"/>
@@ -618,13 +616,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="6"/>
@@ -632,13 +630,13 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="7"/>
@@ -646,13 +644,13 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="6"/>
@@ -660,13 +658,13 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="7"/>
@@ -674,13 +672,13 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="6"/>
@@ -688,13 +686,13 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="7"/>
@@ -702,13 +700,13 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="6"/>
@@ -716,13 +714,13 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="7"/>
@@ -730,13 +728,13 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="6"/>
@@ -744,13 +742,13 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="7"/>
@@ -758,13 +756,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="7"/>
@@ -772,13 +770,13 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="6"/>
@@ -786,13 +784,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="7"/>
@@ -800,13 +798,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="6"/>

</xml_diff>